<commit_message>
📊 Línea 141 actualizada
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-09-13.xlsx
+++ b/data/horarios-141-2026-09-13.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,14 +441,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:14:38</t>
+          <t>Última actualización: 11:24:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -665,6 +665,266 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>19</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>32</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>33</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>68</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>73</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>81</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:47</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>84</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>92</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -677,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -690,16 +950,100 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:14:38</t>
+          <t>Última actualización: 11:24:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
-        </is>
-      </c>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Línea</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>CodigoColectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>11:23:31</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>92</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -725,7 +1069,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:14:38</t>
+          <t>Última actualización: 11:24:22</t>
         </is>
       </c>
     </row>

</xml_diff>